<commit_message>
RateLimiter giới hạn băng thông khi truyền file (Task 25)
</commit_message>
<xml_diff>
--- a/DOCX/Task-List.xlsx
+++ b/DOCX/Task-List.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LTM\UDM11-MultiFileDownloader\DOCX\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6404A1CD-3CC7-4429-B14D-450D7B13BB6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58A6FA40-AC86-4048-8F54-81A5C8D0DA54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Task List" sheetId="1" r:id="rId1"/>
@@ -1791,8 +1791,8 @@
       <c r="H28" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="I28" s="13" t="s">
-        <v>97</v>
+      <c r="I28" s="13">
+        <v>0.6</v>
       </c>
     </row>
     <row r="29" spans="2:9" ht="45" x14ac:dyDescent="0.2">
@@ -1815,7 +1815,9 @@
       <c r="H29" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="I29" s="13"/>
+      <c r="I29" s="13" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="30" spans="2:9" ht="30" x14ac:dyDescent="0.2">
       <c r="B30" s="8">
@@ -1837,7 +1839,9 @@
       <c r="H30" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="I30" s="13"/>
+      <c r="I30" s="13">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="31" spans="2:9" ht="30" x14ac:dyDescent="0.2">
       <c r="B31" s="8">
@@ -1859,7 +1863,9 @@
       <c r="H31" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="I31" s="13"/>
+      <c r="I31" s="13">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="32" spans="2:9" ht="30" x14ac:dyDescent="0.2">
       <c r="B32" s="8">
@@ -1881,7 +1887,9 @@
       <c r="H32" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="I32" s="14"/>
+      <c r="I32" s="14">
+        <v>0.8</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="I6:I32">

</xml_diff>

<commit_message>
feat: Tich hop toan bo du an chay hoan chinh (merge duongkhoa + noi cac module)
- Merge nhanh duongkhoa: UI keo-tha, 2 bang, trang thai ket noi, non-blocking
- Noi DownloadManager: hang doi 3 luong, FileSaver, tien trinh/toc do, doi ten file trung, cach ly loi
- Noi xac thuc SHA-256 sau khi tai (FileIntegrityVerifier)
- Them mau nen trang thai, cot STT, dong thong ke file
- Tach SocketTimeoutManager cho Server
- Khoi phuc entry point Program.cs, sua loi khoi dong GUI
</commit_message>
<xml_diff>
--- a/DOCX/Task-List.xlsx
+++ b/DOCX/Task-List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LTM\UDM11-MultiFileDownloader\DOCX\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58A6FA40-AC86-4048-8F54-81A5C8D0DA54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFC0E4B5-F77D-4256-B9A8-272857BD0D06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="31245" yWindow="840" windowWidth="21600" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Task List" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="104">
   <si>
     <t>STT</t>
   </si>
@@ -415,7 +415,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -512,23 +512,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -567,9 +556,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1204,16 +1190,16 @@
   <dimension ref="B5:AI32"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5" style="15" customWidth="1"/>
-    <col min="2" max="2" width="10.28515625" style="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="39.7109375" style="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="73" style="15" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.7109375" style="15" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.85546875" style="15" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.140625" style="15" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="93.28515625" style="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.5703125" style="15" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="12.5703125" style="15"/>
+    <col min="1" max="1" width="5" style="14" customWidth="1"/>
+    <col min="2" max="2" width="10.28515625" style="14" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39.7109375" style="14" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="73" style="14" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" style="14" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.85546875" style="14" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.140625" style="14" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="93.28515625" style="14" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.5703125" style="14" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="12.5703125" style="14"/>
   </cols>
   <sheetData>
     <row r="5" spans="2:35" x14ac:dyDescent="0.2">
@@ -1267,10 +1253,10 @@
       <c r="H6" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="I6" s="13">
-        <v>0.4</v>
-      </c>
-      <c r="AI6" s="16">
+      <c r="I6" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="AI6" s="15">
         <v>0</v>
       </c>
     </row>
@@ -1297,9 +1283,9 @@
         <v>88</v>
       </c>
       <c r="I7" s="13" t="s">
-        <v>98</v>
-      </c>
-      <c r="AI7" s="16">
+        <v>97</v>
+      </c>
+      <c r="AI7" s="15">
         <v>0.2</v>
       </c>
     </row>
@@ -1328,7 +1314,7 @@
       <c r="I8" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="AI8" s="16">
+      <c r="AI8" s="15">
         <v>0.4</v>
       </c>
     </row>
@@ -1354,8 +1340,10 @@
       <c r="H9" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="I9" s="13"/>
-      <c r="AI9" s="16">
+      <c r="I9" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="AI9" s="15">
         <v>0.6</v>
       </c>
     </row>
@@ -1381,8 +1369,10 @@
       <c r="H10" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="I10" s="13"/>
-      <c r="AI10" s="16">
+      <c r="I10" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="AI10" s="15">
         <v>0.8</v>
       </c>
     </row>
@@ -1408,8 +1398,10 @@
       <c r="H11" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="I11" s="14"/>
-      <c r="AI11" s="16">
+      <c r="I11" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="AI11" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1424,7 +1416,7 @@
         <v>11</v>
       </c>
       <c r="E12" s="4"/>
-      <c r="F12" s="17" t="s">
+      <c r="F12" s="16" t="s">
         <v>100</v>
       </c>
       <c r="G12" s="1" t="s">
@@ -1433,7 +1425,9 @@
       <c r="H12" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="I12" s="13"/>
+      <c r="I12" s="13" t="s">
+        <v>97</v>
+      </c>
       <c r="AI12" s="7" t="s">
         <v>97</v>
       </c>
@@ -1449,7 +1443,7 @@
         <v>22</v>
       </c>
       <c r="E13" s="4"/>
-      <c r="F13" s="17" t="s">
+      <c r="F13" s="16" t="s">
         <v>100</v>
       </c>
       <c r="G13" s="1" t="s">
@@ -1458,8 +1452,10 @@
       <c r="H13" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="I13" s="13"/>
-      <c r="AI13" s="15" t="s">
+      <c r="I13" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="AI13" s="14" t="s">
         <v>99</v>
       </c>
     </row>
@@ -1474,7 +1470,7 @@
         <v>32</v>
       </c>
       <c r="E14" s="4"/>
-      <c r="F14" s="17" t="s">
+      <c r="F14" s="16" t="s">
         <v>100</v>
       </c>
       <c r="G14" s="1" t="s">
@@ -1483,7 +1479,9 @@
       <c r="H14" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="I14" s="13"/>
+      <c r="I14" s="13" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="15" spans="2:35" ht="45" x14ac:dyDescent="0.2">
       <c r="B15" s="8">
@@ -1496,7 +1494,7 @@
         <v>41</v>
       </c>
       <c r="E15" s="4"/>
-      <c r="F15" s="17" t="s">
+      <c r="F15" s="16" t="s">
         <v>100</v>
       </c>
       <c r="G15" s="1" t="s">
@@ -1505,7 +1503,9 @@
       <c r="H15" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="I15" s="13"/>
+      <c r="I15" s="13" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="16" spans="2:35" ht="45" x14ac:dyDescent="0.2">
       <c r="B16" s="8">
@@ -1518,7 +1518,7 @@
         <v>47</v>
       </c>
       <c r="E16" s="4"/>
-      <c r="F16" s="17" t="s">
+      <c r="F16" s="16" t="s">
         <v>100</v>
       </c>
       <c r="G16" s="1" t="s">
@@ -1527,7 +1527,9 @@
       <c r="H16" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="I16" s="14"/>
+      <c r="I16" s="13" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="17" spans="2:9" ht="30" x14ac:dyDescent="0.2">
       <c r="B17" s="8">
@@ -1540,7 +1542,7 @@
         <v>9</v>
       </c>
       <c r="E17" s="4"/>
-      <c r="F17" s="18" t="s">
+      <c r="F17" s="17" t="s">
         <v>101</v>
       </c>
       <c r="G17" s="1" t="s">
@@ -1549,7 +1551,9 @@
       <c r="H17" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="I17" s="13"/>
+      <c r="I17" s="13" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="18" spans="2:9" ht="30" x14ac:dyDescent="0.2">
       <c r="B18" s="8">
@@ -1562,7 +1566,7 @@
         <v>18</v>
       </c>
       <c r="E18" s="4"/>
-      <c r="F18" s="18" t="s">
+      <c r="F18" s="17" t="s">
         <v>101</v>
       </c>
       <c r="G18" s="1" t="s">
@@ -1571,7 +1575,9 @@
       <c r="H18" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="I18" s="13"/>
+      <c r="I18" s="13" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="19" spans="2:9" ht="45" x14ac:dyDescent="0.2">
       <c r="B19" s="8">
@@ -1584,7 +1590,7 @@
         <v>25</v>
       </c>
       <c r="E19" s="4"/>
-      <c r="F19" s="18" t="s">
+      <c r="F19" s="17" t="s">
         <v>101</v>
       </c>
       <c r="G19" s="1" t="s">
@@ -1593,7 +1599,9 @@
       <c r="H19" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="I19" s="13"/>
+      <c r="I19" s="13" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="20" spans="2:9" ht="30" x14ac:dyDescent="0.2">
       <c r="B20" s="8">
@@ -1606,7 +1614,7 @@
         <v>36</v>
       </c>
       <c r="E20" s="4"/>
-      <c r="F20" s="18" t="s">
+      <c r="F20" s="17" t="s">
         <v>101</v>
       </c>
       <c r="G20" s="1" t="s">
@@ -1615,7 +1623,9 @@
       <c r="H20" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="I20" s="13"/>
+      <c r="I20" s="13" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="21" spans="2:9" ht="45" x14ac:dyDescent="0.2">
       <c r="B21" s="8">
@@ -1628,7 +1638,7 @@
         <v>44</v>
       </c>
       <c r="E21" s="4"/>
-      <c r="F21" s="18" t="s">
+      <c r="F21" s="17" t="s">
         <v>101</v>
       </c>
       <c r="G21" s="1" t="s">
@@ -1637,7 +1647,9 @@
       <c r="H21" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="I21" s="14"/>
+      <c r="I21" s="13" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="22" spans="2:9" ht="45" x14ac:dyDescent="0.2">
       <c r="B22" s="8">
@@ -1650,7 +1662,7 @@
         <v>58</v>
       </c>
       <c r="E22" s="4"/>
-      <c r="F22" s="19" t="s">
+      <c r="F22" s="18" t="s">
         <v>103</v>
       </c>
       <c r="G22" s="1" t="s">
@@ -1659,7 +1671,9 @@
       <c r="H22" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="I22" s="13"/>
+      <c r="I22" s="13" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="23" spans="2:9" ht="45" x14ac:dyDescent="0.2">
       <c r="B23" s="8">
@@ -1672,7 +1686,7 @@
         <v>61</v>
       </c>
       <c r="E23" s="4"/>
-      <c r="F23" s="19" t="s">
+      <c r="F23" s="18" t="s">
         <v>103</v>
       </c>
       <c r="G23" s="1" t="s">
@@ -1681,7 +1695,9 @@
       <c r="H23" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="I23" s="13"/>
+      <c r="I23" s="13" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="24" spans="2:9" ht="45" x14ac:dyDescent="0.2">
       <c r="B24" s="8">
@@ -1694,7 +1710,7 @@
         <v>64</v>
       </c>
       <c r="E24" s="4"/>
-      <c r="F24" s="19" t="s">
+      <c r="F24" s="18" t="s">
         <v>103</v>
       </c>
       <c r="G24" s="1" t="s">
@@ -1703,7 +1719,9 @@
       <c r="H24" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="I24" s="13"/>
+      <c r="I24" s="13" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="25" spans="2:9" ht="45" x14ac:dyDescent="0.2">
       <c r="B25" s="8">
@@ -1716,7 +1734,7 @@
         <v>67</v>
       </c>
       <c r="E25" s="4"/>
-      <c r="F25" s="19" t="s">
+      <c r="F25" s="18" t="s">
         <v>103</v>
       </c>
       <c r="G25" s="1" t="s">
@@ -1725,7 +1743,9 @@
       <c r="H25" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="I25" s="13"/>
+      <c r="I25" s="13" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="26" spans="2:9" ht="45" x14ac:dyDescent="0.2">
       <c r="B26" s="8">
@@ -1738,7 +1758,7 @@
         <v>70</v>
       </c>
       <c r="E26" s="4"/>
-      <c r="F26" s="19" t="s">
+      <c r="F26" s="18" t="s">
         <v>103</v>
       </c>
       <c r="G26" s="1" t="s">
@@ -1747,7 +1767,9 @@
       <c r="H26" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="I26" s="14"/>
+      <c r="I26" s="13" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="27" spans="2:9" ht="30" x14ac:dyDescent="0.2">
       <c r="B27" s="8">
@@ -1760,7 +1782,7 @@
         <v>37</v>
       </c>
       <c r="E27" s="4"/>
-      <c r="F27" s="20" t="s">
+      <c r="F27" s="19" t="s">
         <v>102</v>
       </c>
       <c r="G27" s="1" t="s">
@@ -1769,7 +1791,9 @@
       <c r="H27" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="I27" s="13"/>
+      <c r="I27" s="13" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="28" spans="2:9" ht="45" x14ac:dyDescent="0.2">
       <c r="B28" s="8">
@@ -1782,7 +1806,7 @@
         <v>73</v>
       </c>
       <c r="E28" s="4"/>
-      <c r="F28" s="20" t="s">
+      <c r="F28" s="19" t="s">
         <v>102</v>
       </c>
       <c r="G28" s="1" t="s">
@@ -1791,8 +1815,8 @@
       <c r="H28" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="I28" s="13">
-        <v>0.6</v>
+      <c r="I28" s="13" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="29" spans="2:9" ht="45" x14ac:dyDescent="0.2">
@@ -1806,7 +1830,7 @@
         <v>76</v>
       </c>
       <c r="E29" s="4"/>
-      <c r="F29" s="20" t="s">
+      <c r="F29" s="19" t="s">
         <v>102</v>
       </c>
       <c r="G29" s="1" t="s">
@@ -1830,7 +1854,7 @@
         <v>79</v>
       </c>
       <c r="E30" s="4"/>
-      <c r="F30" s="20" t="s">
+      <c r="F30" s="19" t="s">
         <v>102</v>
       </c>
       <c r="G30" s="1" t="s">
@@ -1839,8 +1863,8 @@
       <c r="H30" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="I30" s="13">
-        <v>0.8</v>
+      <c r="I30" s="13" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="31" spans="2:9" ht="30" x14ac:dyDescent="0.2">
@@ -1854,7 +1878,7 @@
         <v>82</v>
       </c>
       <c r="E31" s="4"/>
-      <c r="F31" s="20" t="s">
+      <c r="F31" s="19" t="s">
         <v>102</v>
       </c>
       <c r="G31" s="1" t="s">
@@ -1863,8 +1887,8 @@
       <c r="H31" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="I31" s="13">
-        <v>0.8</v>
+      <c r="I31" s="13" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="32" spans="2:9" ht="30" x14ac:dyDescent="0.2">
@@ -1878,7 +1902,7 @@
         <v>85</v>
       </c>
       <c r="E32" s="4"/>
-      <c r="F32" s="20" t="s">
+      <c r="F32" s="19" t="s">
         <v>102</v>
       </c>
       <c r="G32" s="1" t="s">
@@ -1887,8 +1911,8 @@
       <c r="H32" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="I32" s="14">
-        <v>0.8</v>
+      <c r="I32" s="13" t="s">
+        <v>97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>